<commit_message>
fix: Adição do gráfico de faturamento X produção, além de deixar o gráfico mais visual
</commit_message>
<xml_diff>
--- a/DadosProducao.xlsx
+++ b/DadosProducao.xlsx
@@ -8,16 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pedro.andrade\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{113ADB9C-CD37-4C91-A4C2-134B349713B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5988004-E360-452C-993D-68757E56D6F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16284" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{3AA6C56D-DA97-499B-A05C-D9170B04DAB1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="3" xr2:uid="{3AA6C56D-DA97-499B-A05C-D9170B04DAB1}"/>
   </bookViews>
   <sheets>
     <sheet name="DadosBrutos" sheetId="1" r:id="rId1"/>
     <sheet name="LimpezaDados" sheetId="2" r:id="rId2"/>
+    <sheet name="DadosBacklogXSaudavel" sheetId="3" r:id="rId3"/>
+    <sheet name="DadosFaturamento" sheetId="4" r:id="rId4"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId3"/>
+    <externalReference r:id="rId5"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -61,7 +63,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -83,7 +85,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3007" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3010" uniqueCount="109">
   <si>
     <t>PV</t>
   </si>
@@ -402,12 +404,22 @@
   <si>
     <t>Quantidade</t>
   </si>
+  <si>
+    <t>Saudavel</t>
+  </si>
+  <si>
+    <t>Backlog</t>
+  </si>
+  <si>
+    <t>Vlr Faturado</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
@@ -511,16 +523,17 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Segoe UI"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Consolas"/>
       <family val="3"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="7">
@@ -687,10 +700,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="14" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -731,17 +745,19 @@
     <xf numFmtId="0" fontId="12" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="14" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="11">
     <dxf>
       <font>
         <b/>
@@ -883,16 +899,6 @@
             <color rgb="FFFFC000"/>
           </stop>
         </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
       </fill>
     </dxf>
     <dxf>
@@ -50418,4 +50424,4560 @@
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76D838BA-A018-4D6D-9819-6D56600DF965}">
+  <dimension ref="A1:C727"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="23" t="str" cm="1">
+        <f t="array" ref="A1:A11">_xlfn.UNIQUE(DadosBrutos!C1:C727)</f>
+        <v>DATA</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1" s="23" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="24">
+        <v>46304</v>
+      </c>
+      <c r="B2">
+        <f>COUNTIFS(DadosBrutos!C:C, A2, DadosBrutos!G:G, "SAUDAVEL")</f>
+        <v>6</v>
+      </c>
+      <c r="C2">
+        <f>COUNTIFS(DadosBrutos!C:C, A2, DadosBrutos!G:G, "BACKLOG")</f>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="24">
+        <v>46303</v>
+      </c>
+      <c r="B3">
+        <f>COUNTIFS(DadosBrutos!C:C, A3, DadosBrutos!G:G, "SAUDAVEL")</f>
+        <v>40</v>
+      </c>
+      <c r="C3">
+        <f>COUNTIFS(DadosBrutos!C:C, A3, DadosBrutos!G:G, "BACKLOG")</f>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="24">
+        <v>46302</v>
+      </c>
+      <c r="B4">
+        <f>COUNTIFS(DadosBrutos!C:C, A4, DadosBrutos!G:G, "SAUDAVEL")</f>
+        <v>18</v>
+      </c>
+      <c r="C4">
+        <f>COUNTIFS(DadosBrutos!C:C, A4, DadosBrutos!G:G, "BACKLOG")</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="24">
+        <v>46308</v>
+      </c>
+      <c r="B5">
+        <f>COUNTIFS(DadosBrutos!C:C, A5, DadosBrutos!G:G, "SAUDAVEL")</f>
+        <v>89</v>
+      </c>
+      <c r="C5">
+        <f>COUNTIFS(DadosBrutos!C:C, A5, DadosBrutos!G:G, "BACKLOG")</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="24">
+        <v>46311</v>
+      </c>
+      <c r="B6">
+        <f>COUNTIFS(DadosBrutos!C:C, A6, DadosBrutos!G:G, "SAUDAVEL")</f>
+        <v>27</v>
+      </c>
+      <c r="C6">
+        <f>COUNTIFS(DadosBrutos!C:C, A6, DadosBrutos!G:G, "BACKLOG")</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="24">
+        <v>46307</v>
+      </c>
+      <c r="B7">
+        <f>COUNTIFS(DadosBrutos!C:C, A7, DadosBrutos!G:G, "SAUDAVEL")</f>
+        <v>25</v>
+      </c>
+      <c r="C7">
+        <f>COUNTIFS(DadosBrutos!C:C, A7, DadosBrutos!G:G, "BACKLOG")</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="24">
+        <v>46306</v>
+      </c>
+      <c r="B8">
+        <f>COUNTIFS(DadosBrutos!C:C, A8, DadosBrutos!G:G, "SAUDAVEL")</f>
+        <v>7</v>
+      </c>
+      <c r="C8">
+        <f>COUNTIFS(DadosBrutos!C:C, A8, DadosBrutos!G:G, "BACKLOG")</f>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="24">
+        <v>46305</v>
+      </c>
+      <c r="B9">
+        <f>COUNTIFS(DadosBrutos!C:C, A9, DadosBrutos!G:G, "SAUDAVEL")</f>
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <f>COUNTIFS(DadosBrutos!C:C, A9, DadosBrutos!G:G, "BACKLOG")</f>
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="24">
+        <v>46309</v>
+      </c>
+      <c r="B10">
+        <f>COUNTIFS(DadosBrutos!C:C, A10, DadosBrutos!G:G, "SAUDAVEL")</f>
+        <v>22</v>
+      </c>
+      <c r="C10">
+        <f>COUNTIFS(DadosBrutos!C:C, A10, DadosBrutos!G:G, "BACKLOG")</f>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="24">
+        <v>46310</v>
+      </c>
+      <c r="B11">
+        <f>COUNTIFS(DadosBrutos!C:C, A11, DadosBrutos!G:G, "SAUDAVEL")</f>
+        <v>47</v>
+      </c>
+      <c r="C11">
+        <f>COUNTIFS(DadosBrutos!C:C, A11, DadosBrutos!G:G, "BACKLOG")</f>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="24"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="24"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="24"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="24"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="24"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="24"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="24"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="24"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="24"/>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="24"/>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="24"/>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="24"/>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="24"/>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="24"/>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="24"/>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="24"/>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="24"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="24"/>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="24"/>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="24"/>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="24"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="24"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="24"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="24"/>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="24"/>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="24"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="24"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="24"/>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="24"/>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="24"/>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="24"/>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="24"/>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="24"/>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="24"/>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="24"/>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="24"/>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="24"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="24"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="24"/>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="24"/>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" s="24"/>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="24"/>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="24"/>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="24"/>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="24"/>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="24"/>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="24"/>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="24"/>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="24"/>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" s="24"/>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="24"/>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="24"/>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" s="24"/>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="24"/>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" s="24"/>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" s="24"/>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="24"/>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" s="24"/>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" s="24"/>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" s="24"/>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" s="24"/>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" s="24"/>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" s="24"/>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" s="24"/>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" s="24"/>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" s="24"/>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" s="24"/>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" s="24"/>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" s="24"/>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" s="24"/>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" s="24"/>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" s="24"/>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" s="24"/>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" s="24"/>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" s="24"/>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" s="24"/>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" s="24"/>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" s="24"/>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" s="24"/>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" s="24"/>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" s="24"/>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" s="24"/>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" s="24"/>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" s="24"/>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" s="24"/>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" s="24"/>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" s="24"/>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" s="24"/>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" s="24"/>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" s="24"/>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" s="24"/>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" s="24"/>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104" s="24"/>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105" s="24"/>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106" s="24"/>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A107" s="24"/>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A108" s="24"/>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A109" s="24"/>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A110" s="24"/>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A111" s="24"/>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A112" s="24"/>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A113" s="24"/>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114" s="24"/>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A115" s="24"/>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A116" s="24"/>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117" s="24"/>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118" s="24"/>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A119" s="24"/>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120" s="24"/>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A121" s="24"/>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122" s="24"/>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" s="24"/>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124" s="24"/>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125" s="24"/>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126" s="24"/>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127" s="24"/>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A128" s="24"/>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A129" s="24"/>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A130" s="24"/>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A131" s="24"/>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A132" s="24"/>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A133" s="24"/>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A134" s="24"/>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A135" s="24"/>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A136" s="24"/>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A137" s="24"/>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A138" s="24"/>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A139" s="24"/>
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A140" s="24"/>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A141" s="24"/>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A142" s="24"/>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A143" s="24"/>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A144" s="24"/>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A145" s="24"/>
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A146" s="24"/>
+    </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A147" s="24"/>
+    </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A148" s="24"/>
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A149" s="24"/>
+    </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A150" s="24"/>
+    </row>
+    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A151" s="24"/>
+    </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A152" s="24"/>
+    </row>
+    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A153" s="24"/>
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A154" s="24"/>
+    </row>
+    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A155" s="24"/>
+    </row>
+    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A156" s="24"/>
+    </row>
+    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A157" s="24"/>
+    </row>
+    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A158" s="24"/>
+    </row>
+    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A159" s="24"/>
+    </row>
+    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A160" s="24"/>
+    </row>
+    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A161" s="24"/>
+    </row>
+    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A162" s="24"/>
+    </row>
+    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A163" s="24"/>
+    </row>
+    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A164" s="24"/>
+    </row>
+    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A165" s="24"/>
+    </row>
+    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A166" s="24"/>
+    </row>
+    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A167" s="24"/>
+    </row>
+    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A168" s="24"/>
+    </row>
+    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A169" s="24"/>
+    </row>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A170" s="24"/>
+    </row>
+    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A171" s="24"/>
+    </row>
+    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A172" s="24"/>
+    </row>
+    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A173" s="24"/>
+    </row>
+    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A174" s="24"/>
+    </row>
+    <row r="175" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A175" s="24"/>
+    </row>
+    <row r="176" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A176" s="24"/>
+    </row>
+    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A177" s="24"/>
+    </row>
+    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A178" s="24"/>
+    </row>
+    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A179" s="24"/>
+    </row>
+    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A180" s="24"/>
+    </row>
+    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A181" s="24"/>
+    </row>
+    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A182" s="24"/>
+    </row>
+    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A183" s="24"/>
+    </row>
+    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A184" s="24"/>
+    </row>
+    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A185" s="24"/>
+    </row>
+    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A186" s="24"/>
+    </row>
+    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A187" s="24"/>
+    </row>
+    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A188" s="24"/>
+    </row>
+    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A189" s="24"/>
+    </row>
+    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A190" s="24"/>
+    </row>
+    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A191" s="24"/>
+    </row>
+    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A192" s="24"/>
+    </row>
+    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A193" s="24"/>
+    </row>
+    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A194" s="24"/>
+    </row>
+    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A195" s="24"/>
+    </row>
+    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A196" s="24"/>
+    </row>
+    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A197" s="24"/>
+    </row>
+    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A198" s="24"/>
+    </row>
+    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A199" s="24"/>
+    </row>
+    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A200" s="24"/>
+    </row>
+    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A201" s="24"/>
+    </row>
+    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A202" s="24"/>
+    </row>
+    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A203" s="24"/>
+    </row>
+    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A204" s="24"/>
+    </row>
+    <row r="205" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A205" s="24"/>
+    </row>
+    <row r="206" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A206" s="24"/>
+    </row>
+    <row r="207" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A207" s="24"/>
+    </row>
+    <row r="208" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A208" s="24"/>
+    </row>
+    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A209" s="24"/>
+    </row>
+    <row r="210" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A210" s="24"/>
+    </row>
+    <row r="211" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A211" s="24"/>
+    </row>
+    <row r="212" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A212" s="24"/>
+    </row>
+    <row r="213" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A213" s="24"/>
+    </row>
+    <row r="214" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A214" s="24"/>
+    </row>
+    <row r="215" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A215" s="24"/>
+    </row>
+    <row r="216" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A216" s="24"/>
+    </row>
+    <row r="217" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A217" s="24"/>
+    </row>
+    <row r="218" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A218" s="24"/>
+    </row>
+    <row r="219" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A219" s="24"/>
+    </row>
+    <row r="220" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A220" s="24"/>
+    </row>
+    <row r="221" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A221" s="24"/>
+    </row>
+    <row r="222" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A222" s="24"/>
+    </row>
+    <row r="223" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A223" s="24"/>
+    </row>
+    <row r="224" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A224" s="24"/>
+    </row>
+    <row r="225" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A225" s="24"/>
+    </row>
+    <row r="226" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A226" s="24"/>
+    </row>
+    <row r="227" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A227" s="24"/>
+    </row>
+    <row r="228" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A228" s="24"/>
+    </row>
+    <row r="229" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A229" s="24"/>
+    </row>
+    <row r="230" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A230" s="24"/>
+    </row>
+    <row r="231" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A231" s="24"/>
+    </row>
+    <row r="232" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A232" s="24"/>
+    </row>
+    <row r="233" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A233" s="24"/>
+    </row>
+    <row r="234" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A234" s="24"/>
+    </row>
+    <row r="235" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A235" s="24"/>
+    </row>
+    <row r="236" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A236" s="24"/>
+    </row>
+    <row r="237" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A237" s="24"/>
+    </row>
+    <row r="238" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A238" s="24"/>
+    </row>
+    <row r="239" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A239" s="24"/>
+    </row>
+    <row r="240" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A240" s="24"/>
+    </row>
+    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A241" s="24"/>
+    </row>
+    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A242" s="24"/>
+    </row>
+    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A243" s="24"/>
+    </row>
+    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A244" s="24"/>
+    </row>
+    <row r="245" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A245" s="24"/>
+    </row>
+    <row r="246" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A246" s="24"/>
+    </row>
+    <row r="247" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A247" s="24"/>
+    </row>
+    <row r="248" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A248" s="24"/>
+    </row>
+    <row r="249" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A249" s="24"/>
+    </row>
+    <row r="250" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A250" s="24"/>
+    </row>
+    <row r="251" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A251" s="24"/>
+    </row>
+    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A252" s="24"/>
+    </row>
+    <row r="253" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A253" s="24"/>
+    </row>
+    <row r="254" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A254" s="24"/>
+    </row>
+    <row r="255" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A255" s="24"/>
+    </row>
+    <row r="256" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A256" s="24"/>
+    </row>
+    <row r="257" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A257" s="24"/>
+    </row>
+    <row r="258" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A258" s="24"/>
+    </row>
+    <row r="259" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A259" s="24"/>
+    </row>
+    <row r="260" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A260" s="24"/>
+    </row>
+    <row r="261" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A261" s="24"/>
+    </row>
+    <row r="262" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A262" s="24"/>
+    </row>
+    <row r="263" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A263" s="24"/>
+    </row>
+    <row r="264" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A264" s="24"/>
+    </row>
+    <row r="265" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A265" s="24"/>
+    </row>
+    <row r="266" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A266" s="24"/>
+    </row>
+    <row r="267" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A267" s="24"/>
+    </row>
+    <row r="268" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A268" s="24"/>
+    </row>
+    <row r="269" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A269" s="24"/>
+    </row>
+    <row r="270" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A270" s="24"/>
+    </row>
+    <row r="271" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A271" s="24"/>
+    </row>
+    <row r="272" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A272" s="24"/>
+    </row>
+    <row r="273" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A273" s="24"/>
+    </row>
+    <row r="274" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A274" s="24"/>
+    </row>
+    <row r="275" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A275" s="24"/>
+    </row>
+    <row r="276" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A276" s="24"/>
+    </row>
+    <row r="277" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A277" s="24"/>
+    </row>
+    <row r="278" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A278" s="24"/>
+    </row>
+    <row r="279" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A279" s="24"/>
+    </row>
+    <row r="280" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A280" s="24"/>
+    </row>
+    <row r="281" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A281" s="24"/>
+    </row>
+    <row r="282" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A282" s="24"/>
+    </row>
+    <row r="283" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A283" s="24"/>
+    </row>
+    <row r="284" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A284" s="24"/>
+    </row>
+    <row r="285" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A285" s="24"/>
+    </row>
+    <row r="286" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A286" s="24"/>
+    </row>
+    <row r="287" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A287" s="24"/>
+    </row>
+    <row r="288" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A288" s="24"/>
+    </row>
+    <row r="289" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A289" s="24"/>
+    </row>
+    <row r="290" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A290" s="24"/>
+    </row>
+    <row r="291" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A291" s="24"/>
+    </row>
+    <row r="292" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A292" s="24"/>
+    </row>
+    <row r="293" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A293" s="24"/>
+    </row>
+    <row r="294" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A294" s="24"/>
+    </row>
+    <row r="295" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A295" s="24"/>
+    </row>
+    <row r="296" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A296" s="24"/>
+    </row>
+    <row r="297" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A297" s="24"/>
+    </row>
+    <row r="298" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A298" s="24"/>
+    </row>
+    <row r="299" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A299" s="24"/>
+    </row>
+    <row r="300" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A300" s="24"/>
+    </row>
+    <row r="301" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A301" s="24"/>
+    </row>
+    <row r="302" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A302" s="24"/>
+    </row>
+    <row r="303" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A303" s="24"/>
+    </row>
+    <row r="304" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A304" s="24"/>
+    </row>
+    <row r="305" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A305" s="24"/>
+    </row>
+    <row r="306" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A306" s="24"/>
+    </row>
+    <row r="307" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A307" s="24"/>
+    </row>
+    <row r="308" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A308" s="24"/>
+    </row>
+    <row r="309" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A309" s="24"/>
+    </row>
+    <row r="310" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A310" s="24"/>
+    </row>
+    <row r="311" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A311" s="24"/>
+    </row>
+    <row r="312" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A312" s="24"/>
+    </row>
+    <row r="313" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A313" s="24"/>
+    </row>
+    <row r="314" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A314" s="24"/>
+    </row>
+    <row r="315" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A315" s="24"/>
+    </row>
+    <row r="316" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A316" s="24"/>
+    </row>
+    <row r="317" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A317" s="24"/>
+    </row>
+    <row r="318" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A318" s="24"/>
+    </row>
+    <row r="319" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A319" s="24"/>
+    </row>
+    <row r="320" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A320" s="24"/>
+    </row>
+    <row r="321" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A321" s="24"/>
+    </row>
+    <row r="322" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A322" s="24"/>
+    </row>
+    <row r="323" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A323" s="24"/>
+    </row>
+    <row r="324" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A324" s="24"/>
+    </row>
+    <row r="325" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A325" s="24"/>
+    </row>
+    <row r="326" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A326" s="24"/>
+    </row>
+    <row r="327" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A327" s="24"/>
+    </row>
+    <row r="328" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A328" s="24"/>
+    </row>
+    <row r="329" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A329" s="24"/>
+    </row>
+    <row r="330" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A330" s="24"/>
+    </row>
+    <row r="331" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A331" s="24"/>
+    </row>
+    <row r="332" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A332" s="24"/>
+    </row>
+    <row r="333" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A333" s="24"/>
+    </row>
+    <row r="334" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A334" s="24"/>
+    </row>
+    <row r="335" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A335" s="24"/>
+    </row>
+    <row r="336" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A336" s="24"/>
+    </row>
+    <row r="337" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A337" s="24"/>
+    </row>
+    <row r="338" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A338" s="24"/>
+    </row>
+    <row r="339" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A339" s="24"/>
+    </row>
+    <row r="340" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A340" s="24"/>
+    </row>
+    <row r="341" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A341" s="24"/>
+    </row>
+    <row r="342" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A342" s="24"/>
+    </row>
+    <row r="343" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A343" s="24"/>
+    </row>
+    <row r="344" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A344" s="24"/>
+    </row>
+    <row r="345" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A345" s="24"/>
+    </row>
+    <row r="346" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A346" s="24"/>
+    </row>
+    <row r="347" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A347" s="24"/>
+    </row>
+    <row r="348" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A348" s="24"/>
+    </row>
+    <row r="349" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A349" s="24"/>
+    </row>
+    <row r="350" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A350" s="24"/>
+    </row>
+    <row r="351" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A351" s="24"/>
+    </row>
+    <row r="352" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A352" s="24"/>
+    </row>
+    <row r="353" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A353" s="24"/>
+    </row>
+    <row r="354" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A354" s="24"/>
+    </row>
+    <row r="355" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A355" s="24"/>
+    </row>
+    <row r="356" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A356" s="24"/>
+    </row>
+    <row r="357" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A357" s="24"/>
+    </row>
+    <row r="358" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A358" s="24"/>
+    </row>
+    <row r="359" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A359" s="24"/>
+    </row>
+    <row r="360" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A360" s="24"/>
+    </row>
+    <row r="361" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A361" s="24"/>
+    </row>
+    <row r="362" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A362" s="24"/>
+    </row>
+    <row r="363" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A363" s="24"/>
+    </row>
+    <row r="364" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A364" s="24"/>
+    </row>
+    <row r="365" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A365" s="24"/>
+    </row>
+    <row r="366" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A366" s="24"/>
+    </row>
+    <row r="367" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A367" s="24"/>
+    </row>
+    <row r="368" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A368" s="24"/>
+    </row>
+    <row r="369" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A369" s="24"/>
+    </row>
+    <row r="370" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A370" s="24"/>
+    </row>
+    <row r="371" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A371" s="24"/>
+    </row>
+    <row r="372" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A372" s="24"/>
+    </row>
+    <row r="373" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A373" s="24"/>
+    </row>
+    <row r="374" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A374" s="24"/>
+    </row>
+    <row r="375" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A375" s="24"/>
+    </row>
+    <row r="376" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A376" s="24"/>
+    </row>
+    <row r="377" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A377" s="24"/>
+    </row>
+    <row r="378" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A378" s="24"/>
+    </row>
+    <row r="379" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A379" s="24"/>
+    </row>
+    <row r="380" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A380" s="24"/>
+    </row>
+    <row r="381" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A381" s="24"/>
+    </row>
+    <row r="382" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A382" s="24"/>
+    </row>
+    <row r="383" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A383" s="24"/>
+    </row>
+    <row r="384" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A384" s="24"/>
+    </row>
+    <row r="385" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A385" s="24"/>
+    </row>
+    <row r="386" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A386" s="24"/>
+    </row>
+    <row r="387" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A387" s="24"/>
+    </row>
+    <row r="388" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A388" s="24"/>
+    </row>
+    <row r="389" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A389" s="24"/>
+    </row>
+    <row r="390" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A390" s="24"/>
+    </row>
+    <row r="391" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A391" s="24"/>
+    </row>
+    <row r="392" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A392" s="24"/>
+    </row>
+    <row r="393" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A393" s="24"/>
+    </row>
+    <row r="394" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A394" s="24"/>
+    </row>
+    <row r="395" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A395" s="24"/>
+    </row>
+    <row r="396" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A396" s="24"/>
+    </row>
+    <row r="397" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A397" s="24"/>
+    </row>
+    <row r="398" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A398" s="24"/>
+    </row>
+    <row r="399" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A399" s="24"/>
+    </row>
+    <row r="400" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A400" s="24"/>
+    </row>
+    <row r="401" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A401" s="24"/>
+    </row>
+    <row r="402" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A402" s="24"/>
+    </row>
+    <row r="403" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A403" s="24"/>
+    </row>
+    <row r="404" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A404" s="24"/>
+    </row>
+    <row r="405" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A405" s="24"/>
+    </row>
+    <row r="406" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A406" s="24"/>
+    </row>
+    <row r="407" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A407" s="24"/>
+    </row>
+    <row r="408" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A408" s="24"/>
+    </row>
+    <row r="409" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A409" s="24"/>
+    </row>
+    <row r="410" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A410" s="24"/>
+    </row>
+    <row r="411" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A411" s="24"/>
+    </row>
+    <row r="412" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A412" s="24"/>
+    </row>
+    <row r="413" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A413" s="24"/>
+    </row>
+    <row r="414" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A414" s="24"/>
+    </row>
+    <row r="415" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A415" s="24"/>
+    </row>
+    <row r="416" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A416" s="24"/>
+    </row>
+    <row r="417" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A417" s="24"/>
+    </row>
+    <row r="418" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A418" s="24"/>
+    </row>
+    <row r="419" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A419" s="24"/>
+    </row>
+    <row r="420" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A420" s="24"/>
+    </row>
+    <row r="421" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A421" s="24"/>
+    </row>
+    <row r="422" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A422" s="24"/>
+    </row>
+    <row r="423" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A423" s="24"/>
+    </row>
+    <row r="424" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A424" s="24"/>
+    </row>
+    <row r="425" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A425" s="24"/>
+    </row>
+    <row r="426" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A426" s="24"/>
+    </row>
+    <row r="427" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A427" s="24"/>
+    </row>
+    <row r="428" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A428" s="24"/>
+    </row>
+    <row r="429" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A429" s="24"/>
+    </row>
+    <row r="430" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A430" s="24"/>
+    </row>
+    <row r="431" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A431" s="24"/>
+    </row>
+    <row r="432" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A432" s="24"/>
+    </row>
+    <row r="433" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A433" s="24"/>
+    </row>
+    <row r="434" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A434" s="24"/>
+    </row>
+    <row r="435" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A435" s="24"/>
+    </row>
+    <row r="436" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A436" s="24"/>
+    </row>
+    <row r="437" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A437" s="24"/>
+    </row>
+    <row r="438" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A438" s="24"/>
+    </row>
+    <row r="439" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A439" s="24"/>
+    </row>
+    <row r="440" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A440" s="24"/>
+    </row>
+    <row r="441" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A441" s="24"/>
+    </row>
+    <row r="442" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A442" s="24"/>
+    </row>
+    <row r="443" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A443" s="24"/>
+    </row>
+    <row r="444" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A444" s="24"/>
+    </row>
+    <row r="445" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A445" s="24"/>
+    </row>
+    <row r="446" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A446" s="24"/>
+    </row>
+    <row r="447" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A447" s="24"/>
+    </row>
+    <row r="448" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A448" s="24"/>
+    </row>
+    <row r="449" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A449" s="24"/>
+    </row>
+    <row r="450" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A450" s="24"/>
+    </row>
+    <row r="451" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A451" s="24"/>
+    </row>
+    <row r="452" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A452" s="24"/>
+    </row>
+    <row r="453" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A453" s="24"/>
+    </row>
+    <row r="454" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A454" s="24"/>
+    </row>
+    <row r="455" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A455" s="24"/>
+    </row>
+    <row r="456" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A456" s="24"/>
+    </row>
+    <row r="457" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A457" s="24"/>
+    </row>
+    <row r="458" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A458" s="24"/>
+    </row>
+    <row r="459" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A459" s="24"/>
+    </row>
+    <row r="460" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A460" s="24"/>
+    </row>
+    <row r="461" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A461" s="24"/>
+    </row>
+    <row r="462" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A462" s="24"/>
+    </row>
+    <row r="463" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A463" s="24"/>
+    </row>
+    <row r="464" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A464" s="24"/>
+    </row>
+    <row r="465" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A465" s="24"/>
+    </row>
+    <row r="466" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A466" s="24"/>
+    </row>
+    <row r="467" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A467" s="24"/>
+    </row>
+    <row r="468" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A468" s="24"/>
+    </row>
+    <row r="469" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A469" s="24"/>
+    </row>
+    <row r="470" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A470" s="24"/>
+    </row>
+    <row r="471" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A471" s="24"/>
+    </row>
+    <row r="472" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A472" s="24"/>
+    </row>
+    <row r="473" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A473" s="24"/>
+    </row>
+    <row r="474" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A474" s="24"/>
+    </row>
+    <row r="475" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A475" s="24"/>
+    </row>
+    <row r="476" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A476" s="24"/>
+    </row>
+    <row r="477" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A477" s="24"/>
+    </row>
+    <row r="478" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A478" s="24"/>
+    </row>
+    <row r="479" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A479" s="24"/>
+    </row>
+    <row r="480" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A480" s="24"/>
+    </row>
+    <row r="481" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A481" s="24"/>
+    </row>
+    <row r="482" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A482" s="24"/>
+    </row>
+    <row r="483" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A483" s="24"/>
+    </row>
+    <row r="484" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A484" s="24"/>
+    </row>
+    <row r="485" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A485" s="24"/>
+    </row>
+    <row r="486" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A486" s="24"/>
+    </row>
+    <row r="487" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A487" s="24"/>
+    </row>
+    <row r="488" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A488" s="24"/>
+    </row>
+    <row r="489" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A489" s="24"/>
+    </row>
+    <row r="490" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A490" s="24"/>
+    </row>
+    <row r="491" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A491" s="24"/>
+    </row>
+    <row r="492" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A492" s="24"/>
+    </row>
+    <row r="493" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A493" s="24"/>
+    </row>
+    <row r="494" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A494" s="24"/>
+    </row>
+    <row r="495" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A495" s="24"/>
+    </row>
+    <row r="496" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A496" s="24"/>
+    </row>
+    <row r="497" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A497" s="24"/>
+    </row>
+    <row r="498" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A498" s="24"/>
+    </row>
+    <row r="499" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A499" s="24"/>
+    </row>
+    <row r="500" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A500" s="24"/>
+    </row>
+    <row r="501" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A501" s="24"/>
+    </row>
+    <row r="502" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A502" s="24"/>
+    </row>
+    <row r="503" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A503" s="24"/>
+    </row>
+    <row r="504" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A504" s="24"/>
+    </row>
+    <row r="505" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A505" s="24"/>
+    </row>
+    <row r="506" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A506" s="24"/>
+    </row>
+    <row r="507" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A507" s="24"/>
+    </row>
+    <row r="508" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A508" s="24"/>
+    </row>
+    <row r="509" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A509" s="24"/>
+    </row>
+    <row r="510" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A510" s="24"/>
+    </row>
+    <row r="511" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A511" s="24"/>
+    </row>
+    <row r="512" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A512" s="24"/>
+    </row>
+    <row r="513" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A513" s="24"/>
+    </row>
+    <row r="514" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A514" s="24"/>
+    </row>
+    <row r="515" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A515" s="24"/>
+    </row>
+    <row r="516" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A516" s="24"/>
+    </row>
+    <row r="517" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A517" s="24"/>
+    </row>
+    <row r="518" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A518" s="24"/>
+    </row>
+    <row r="519" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A519" s="24"/>
+    </row>
+    <row r="520" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A520" s="24"/>
+    </row>
+    <row r="521" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A521" s="24"/>
+    </row>
+    <row r="522" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A522" s="24"/>
+    </row>
+    <row r="523" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A523" s="24"/>
+    </row>
+    <row r="524" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A524" s="24"/>
+    </row>
+    <row r="525" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A525" s="24"/>
+    </row>
+    <row r="526" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A526" s="24"/>
+    </row>
+    <row r="527" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A527" s="24"/>
+    </row>
+    <row r="528" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A528" s="24"/>
+    </row>
+    <row r="529" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A529" s="24"/>
+    </row>
+    <row r="530" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A530" s="24"/>
+    </row>
+    <row r="531" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A531" s="24"/>
+    </row>
+    <row r="532" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A532" s="24"/>
+    </row>
+    <row r="533" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A533" s="24"/>
+    </row>
+    <row r="534" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A534" s="24"/>
+    </row>
+    <row r="535" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A535" s="24"/>
+    </row>
+    <row r="536" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A536" s="24"/>
+    </row>
+    <row r="537" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A537" s="24"/>
+    </row>
+    <row r="538" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A538" s="24"/>
+    </row>
+    <row r="539" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A539" s="24"/>
+    </row>
+    <row r="540" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A540" s="24"/>
+    </row>
+    <row r="541" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A541" s="24"/>
+    </row>
+    <row r="542" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A542" s="24"/>
+    </row>
+    <row r="543" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A543" s="24"/>
+    </row>
+    <row r="544" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A544" s="24"/>
+    </row>
+    <row r="545" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A545" s="24"/>
+    </row>
+    <row r="546" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A546" s="24"/>
+    </row>
+    <row r="547" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A547" s="24"/>
+    </row>
+    <row r="548" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A548" s="24"/>
+    </row>
+    <row r="549" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A549" s="24"/>
+    </row>
+    <row r="550" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A550" s="24"/>
+    </row>
+    <row r="551" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A551" s="24"/>
+    </row>
+    <row r="552" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A552" s="24"/>
+    </row>
+    <row r="553" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A553" s="24"/>
+    </row>
+    <row r="554" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A554" s="24"/>
+    </row>
+    <row r="555" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A555" s="24"/>
+    </row>
+    <row r="556" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A556" s="24"/>
+    </row>
+    <row r="557" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A557" s="24"/>
+    </row>
+    <row r="558" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A558" s="24"/>
+    </row>
+    <row r="559" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A559" s="24"/>
+    </row>
+    <row r="560" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A560" s="24"/>
+    </row>
+    <row r="561" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A561" s="24"/>
+    </row>
+    <row r="562" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A562" s="24"/>
+    </row>
+    <row r="563" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A563" s="24"/>
+    </row>
+    <row r="564" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A564" s="24"/>
+    </row>
+    <row r="565" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A565" s="24"/>
+    </row>
+    <row r="566" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A566" s="24"/>
+    </row>
+    <row r="567" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A567" s="24"/>
+    </row>
+    <row r="568" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A568" s="24"/>
+    </row>
+    <row r="569" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A569" s="24"/>
+    </row>
+    <row r="570" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A570" s="24"/>
+    </row>
+    <row r="571" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A571" s="24"/>
+    </row>
+    <row r="572" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A572" s="24"/>
+    </row>
+    <row r="573" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A573" s="24"/>
+    </row>
+    <row r="574" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A574" s="24"/>
+    </row>
+    <row r="575" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A575" s="24"/>
+    </row>
+    <row r="576" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A576" s="24"/>
+    </row>
+    <row r="577" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A577" s="24"/>
+    </row>
+    <row r="578" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A578" s="24"/>
+    </row>
+    <row r="579" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A579" s="24"/>
+    </row>
+    <row r="580" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A580" s="24"/>
+    </row>
+    <row r="581" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A581" s="24"/>
+    </row>
+    <row r="582" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A582" s="24"/>
+    </row>
+    <row r="583" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A583" s="24"/>
+    </row>
+    <row r="584" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A584" s="24"/>
+    </row>
+    <row r="585" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A585" s="24"/>
+    </row>
+    <row r="586" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A586" s="24"/>
+    </row>
+    <row r="587" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A587" s="24"/>
+    </row>
+    <row r="588" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A588" s="24"/>
+    </row>
+    <row r="589" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A589" s="24"/>
+    </row>
+    <row r="590" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A590" s="24"/>
+    </row>
+    <row r="591" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A591" s="24"/>
+    </row>
+    <row r="592" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A592" s="24"/>
+    </row>
+    <row r="593" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A593" s="24"/>
+    </row>
+    <row r="594" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A594" s="24"/>
+    </row>
+    <row r="595" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A595" s="24"/>
+    </row>
+    <row r="596" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A596" s="24"/>
+    </row>
+    <row r="597" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A597" s="24"/>
+    </row>
+    <row r="598" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A598" s="24"/>
+    </row>
+    <row r="599" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A599" s="24"/>
+    </row>
+    <row r="600" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A600" s="24"/>
+    </row>
+    <row r="601" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A601" s="24"/>
+    </row>
+    <row r="602" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A602" s="24"/>
+    </row>
+    <row r="603" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A603" s="24"/>
+    </row>
+    <row r="604" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A604" s="24"/>
+    </row>
+    <row r="605" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A605" s="24"/>
+    </row>
+    <row r="606" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A606" s="24"/>
+    </row>
+    <row r="607" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A607" s="24"/>
+    </row>
+    <row r="608" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A608" s="24"/>
+    </row>
+    <row r="609" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A609" s="24"/>
+    </row>
+    <row r="610" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A610" s="24"/>
+    </row>
+    <row r="611" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A611" s="24"/>
+    </row>
+    <row r="612" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A612" s="24"/>
+    </row>
+    <row r="613" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A613" s="24"/>
+    </row>
+    <row r="614" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A614" s="24"/>
+    </row>
+    <row r="615" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A615" s="24"/>
+    </row>
+    <row r="616" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A616" s="24"/>
+    </row>
+    <row r="617" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A617" s="24"/>
+    </row>
+    <row r="618" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A618" s="24"/>
+    </row>
+    <row r="619" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A619" s="24"/>
+    </row>
+    <row r="620" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A620" s="24"/>
+    </row>
+    <row r="621" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A621" s="24"/>
+    </row>
+    <row r="622" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A622" s="24"/>
+    </row>
+    <row r="623" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A623" s="24"/>
+    </row>
+    <row r="624" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A624" s="24"/>
+    </row>
+    <row r="625" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A625" s="24"/>
+    </row>
+    <row r="626" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A626" s="24"/>
+    </row>
+    <row r="627" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A627" s="24"/>
+    </row>
+    <row r="628" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A628" s="24"/>
+    </row>
+    <row r="629" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A629" s="24"/>
+    </row>
+    <row r="630" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A630" s="24"/>
+    </row>
+    <row r="631" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A631" s="24"/>
+    </row>
+    <row r="632" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A632" s="24"/>
+    </row>
+    <row r="633" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A633" s="24"/>
+    </row>
+    <row r="634" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A634" s="24"/>
+    </row>
+    <row r="635" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A635" s="24"/>
+    </row>
+    <row r="636" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A636" s="24"/>
+    </row>
+    <row r="637" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A637" s="24"/>
+    </row>
+    <row r="638" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A638" s="24"/>
+    </row>
+    <row r="639" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A639" s="24"/>
+    </row>
+    <row r="640" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A640" s="24"/>
+    </row>
+    <row r="641" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A641" s="24"/>
+    </row>
+    <row r="642" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A642" s="24"/>
+    </row>
+    <row r="643" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A643" s="24"/>
+    </row>
+    <row r="644" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A644" s="24"/>
+    </row>
+    <row r="645" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A645" s="24"/>
+    </row>
+    <row r="646" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A646" s="24"/>
+    </row>
+    <row r="647" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A647" s="24"/>
+    </row>
+    <row r="648" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A648" s="24"/>
+    </row>
+    <row r="649" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A649" s="24"/>
+    </row>
+    <row r="650" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A650" s="24"/>
+    </row>
+    <row r="651" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A651" s="24"/>
+    </row>
+    <row r="652" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A652" s="24"/>
+    </row>
+    <row r="653" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A653" s="24"/>
+    </row>
+    <row r="654" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A654" s="24"/>
+    </row>
+    <row r="655" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A655" s="24"/>
+    </row>
+    <row r="656" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A656" s="24"/>
+    </row>
+    <row r="657" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A657" s="24"/>
+    </row>
+    <row r="658" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A658" s="24"/>
+    </row>
+    <row r="659" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A659" s="24"/>
+    </row>
+    <row r="660" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A660" s="24"/>
+    </row>
+    <row r="661" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A661" s="24"/>
+    </row>
+    <row r="662" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A662" s="24"/>
+    </row>
+    <row r="663" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A663" s="24"/>
+    </row>
+    <row r="664" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A664" s="24"/>
+    </row>
+    <row r="665" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A665" s="24"/>
+    </row>
+    <row r="666" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A666" s="24"/>
+    </row>
+    <row r="667" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A667" s="24"/>
+    </row>
+    <row r="668" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A668" s="24"/>
+    </row>
+    <row r="669" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A669" s="24"/>
+    </row>
+    <row r="670" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A670" s="24"/>
+    </row>
+    <row r="671" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A671" s="24"/>
+    </row>
+    <row r="672" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A672" s="24"/>
+    </row>
+    <row r="673" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A673" s="24"/>
+    </row>
+    <row r="674" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A674" s="24"/>
+    </row>
+    <row r="675" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A675" s="24"/>
+    </row>
+    <row r="676" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A676" s="24"/>
+    </row>
+    <row r="677" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A677" s="24"/>
+    </row>
+    <row r="678" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A678" s="24"/>
+    </row>
+    <row r="679" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A679" s="24"/>
+    </row>
+    <row r="680" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A680" s="24"/>
+    </row>
+    <row r="681" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A681" s="24"/>
+    </row>
+    <row r="682" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A682" s="24"/>
+    </row>
+    <row r="683" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A683" s="24"/>
+    </row>
+    <row r="684" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A684" s="24"/>
+    </row>
+    <row r="685" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A685" s="25"/>
+    </row>
+    <row r="686" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A686" s="25"/>
+    </row>
+    <row r="687" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A687" s="25"/>
+    </row>
+    <row r="688" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A688" s="25"/>
+    </row>
+    <row r="689" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A689" s="25"/>
+    </row>
+    <row r="690" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A690" s="25"/>
+    </row>
+    <row r="691" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A691" s="25"/>
+    </row>
+    <row r="692" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A692" s="25"/>
+    </row>
+    <row r="693" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A693" s="25"/>
+    </row>
+    <row r="694" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A694" s="25"/>
+    </row>
+    <row r="695" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A695" s="25"/>
+    </row>
+    <row r="696" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A696" s="25"/>
+    </row>
+    <row r="697" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A697" s="25"/>
+    </row>
+    <row r="698" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A698" s="25"/>
+    </row>
+    <row r="699" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A699" s="25"/>
+    </row>
+    <row r="700" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A700" s="25"/>
+    </row>
+    <row r="701" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A701" s="25"/>
+    </row>
+    <row r="702" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A702" s="25"/>
+    </row>
+    <row r="703" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A703" s="25"/>
+    </row>
+    <row r="704" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A704" s="25"/>
+    </row>
+    <row r="705" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A705" s="25"/>
+    </row>
+    <row r="706" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A706" s="25"/>
+    </row>
+    <row r="707" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A707" s="25"/>
+    </row>
+    <row r="708" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A708" s="25"/>
+    </row>
+    <row r="709" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A709" s="25"/>
+    </row>
+    <row r="710" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A710" s="25"/>
+    </row>
+    <row r="711" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A711" s="25"/>
+    </row>
+    <row r="712" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A712" s="25"/>
+    </row>
+    <row r="713" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A713" s="25"/>
+    </row>
+    <row r="714" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A714" s="25"/>
+    </row>
+    <row r="715" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A715" s="25"/>
+    </row>
+    <row r="716" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A716" s="25"/>
+    </row>
+    <row r="717" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A717" s="25"/>
+    </row>
+    <row r="718" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A718" s="25"/>
+    </row>
+    <row r="719" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A719" s="25"/>
+    </row>
+    <row r="720" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A720" s="25"/>
+    </row>
+    <row r="721" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A721" s="25"/>
+    </row>
+    <row r="722" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A722" s="25"/>
+    </row>
+    <row r="723" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A723" s="25"/>
+    </row>
+    <row r="724" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A724" s="25"/>
+    </row>
+    <row r="725" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A725" s="25"/>
+    </row>
+    <row r="726" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A726" s="25"/>
+    </row>
+    <row r="727" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A727" s="25"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A8FB21-A1F8-40C7-9CA7-CA07CB9FFF27}">
+  <dimension ref="A1:B727"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A1" s="23" t="str" cm="1">
+        <f t="array" ref="A1:A11">_xlfn.UNIQUE(DadosBrutos!C1:C727)</f>
+        <v>DATA</v>
+      </c>
+      <c r="B1" s="23" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="24">
+        <v>46304</v>
+      </c>
+      <c r="B2" s="26">
+        <v>323204.13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="24">
+        <v>46303</v>
+      </c>
+      <c r="B3" s="26">
+        <v>766597.26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="24">
+        <v>46302</v>
+      </c>
+      <c r="B4" s="26">
+        <v>322663.09000000003</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="24">
+        <v>46308</v>
+      </c>
+      <c r="B5" s="26">
+        <v>476395.59</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="24">
+        <v>46311</v>
+      </c>
+      <c r="B6" s="26">
+        <v>1395331.97</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="24">
+        <v>46307</v>
+      </c>
+      <c r="B7" s="26">
+        <v>216275.07</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="24">
+        <v>46306</v>
+      </c>
+      <c r="B8" s="26">
+        <v>203448.42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="24">
+        <v>46305</v>
+      </c>
+      <c r="B9" s="26">
+        <v>218825.18</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="24">
+        <v>46309</v>
+      </c>
+      <c r="B10" s="26">
+        <v>329456.51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="24">
+        <v>46310</v>
+      </c>
+      <c r="B11" s="26">
+        <v>300180.06</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="24"/>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="24"/>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="24"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="24"/>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="24"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="24"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="24"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="24"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" s="24"/>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" s="24"/>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="24"/>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="24"/>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="24"/>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="24"/>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="24"/>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="24"/>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="24"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="24"/>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" s="24"/>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" s="24"/>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="24"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="24"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="24"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="24"/>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="24"/>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="24"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="24"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="24"/>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="24"/>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="24"/>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="24"/>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="24"/>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="24"/>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="24"/>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="24"/>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="24"/>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="24"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="24"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="24"/>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="24"/>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" s="24"/>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="24"/>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="24"/>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="24"/>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" s="24"/>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" s="24"/>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="24"/>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="24"/>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="24"/>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" s="24"/>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="24"/>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="24"/>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" s="24"/>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="24"/>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" s="24"/>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" s="24"/>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" s="24"/>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" s="24"/>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" s="24"/>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" s="24"/>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" s="24"/>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" s="24"/>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" s="24"/>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" s="24"/>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" s="24"/>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" s="24"/>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" s="24"/>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" s="24"/>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" s="24"/>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" s="24"/>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" s="24"/>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" s="24"/>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" s="24"/>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" s="24"/>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" s="24"/>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" s="24"/>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" s="24"/>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" s="24"/>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" s="24"/>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" s="24"/>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" s="24"/>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" s="24"/>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" s="24"/>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" s="24"/>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" s="24"/>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" s="24"/>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" s="24"/>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" s="24"/>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" s="24"/>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" s="24"/>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" s="24"/>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" s="24"/>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104" s="24"/>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105" s="24"/>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106" s="24"/>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A107" s="24"/>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A108" s="24"/>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A109" s="24"/>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A110" s="24"/>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A111" s="24"/>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A112" s="24"/>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A113" s="24"/>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114" s="24"/>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A115" s="24"/>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A116" s="24"/>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117" s="24"/>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118" s="24"/>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A119" s="24"/>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120" s="24"/>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A121" s="24"/>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122" s="24"/>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" s="24"/>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124" s="24"/>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125" s="24"/>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126" s="24"/>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127" s="24"/>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A128" s="24"/>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A129" s="24"/>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A130" s="24"/>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A131" s="24"/>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A132" s="24"/>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A133" s="24"/>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A134" s="24"/>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A135" s="24"/>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A136" s="24"/>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A137" s="24"/>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A138" s="24"/>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A139" s="24"/>
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A140" s="24"/>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A141" s="24"/>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A142" s="24"/>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A143" s="24"/>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A144" s="24"/>
+    </row>
+    <row r="145" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A145" s="24"/>
+    </row>
+    <row r="146" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A146" s="24"/>
+    </row>
+    <row r="147" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A147" s="24"/>
+    </row>
+    <row r="148" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A148" s="24"/>
+    </row>
+    <row r="149" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A149" s="24"/>
+    </row>
+    <row r="150" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A150" s="24"/>
+    </row>
+    <row r="151" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A151" s="24"/>
+    </row>
+    <row r="152" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A152" s="24"/>
+    </row>
+    <row r="153" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A153" s="24"/>
+    </row>
+    <row r="154" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A154" s="24"/>
+    </row>
+    <row r="155" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A155" s="24"/>
+    </row>
+    <row r="156" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A156" s="24"/>
+    </row>
+    <row r="157" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A157" s="24"/>
+    </row>
+    <row r="158" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A158" s="24"/>
+    </row>
+    <row r="159" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A159" s="24"/>
+    </row>
+    <row r="160" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A160" s="24"/>
+    </row>
+    <row r="161" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A161" s="24"/>
+    </row>
+    <row r="162" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A162" s="24"/>
+    </row>
+    <row r="163" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A163" s="24"/>
+    </row>
+    <row r="164" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A164" s="24"/>
+    </row>
+    <row r="165" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A165" s="24"/>
+    </row>
+    <row r="166" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A166" s="24"/>
+    </row>
+    <row r="167" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A167" s="24"/>
+    </row>
+    <row r="168" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A168" s="24"/>
+    </row>
+    <row r="169" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A169" s="24"/>
+    </row>
+    <row r="170" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A170" s="24"/>
+    </row>
+    <row r="171" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A171" s="24"/>
+    </row>
+    <row r="172" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A172" s="24"/>
+    </row>
+    <row r="173" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A173" s="24"/>
+    </row>
+    <row r="174" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A174" s="24"/>
+    </row>
+    <row r="175" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A175" s="24"/>
+    </row>
+    <row r="176" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A176" s="24"/>
+    </row>
+    <row r="177" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A177" s="24"/>
+    </row>
+    <row r="178" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A178" s="24"/>
+    </row>
+    <row r="179" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A179" s="24"/>
+    </row>
+    <row r="180" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A180" s="24"/>
+    </row>
+    <row r="181" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A181" s="24"/>
+    </row>
+    <row r="182" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A182" s="24"/>
+    </row>
+    <row r="183" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A183" s="24"/>
+    </row>
+    <row r="184" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A184" s="24"/>
+    </row>
+    <row r="185" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A185" s="24"/>
+    </row>
+    <row r="186" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A186" s="24"/>
+    </row>
+    <row r="187" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A187" s="24"/>
+    </row>
+    <row r="188" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A188" s="24"/>
+    </row>
+    <row r="189" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A189" s="24"/>
+    </row>
+    <row r="190" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A190" s="24"/>
+    </row>
+    <row r="191" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A191" s="24"/>
+    </row>
+    <row r="192" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A192" s="24"/>
+    </row>
+    <row r="193" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A193" s="24"/>
+    </row>
+    <row r="194" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A194" s="24"/>
+    </row>
+    <row r="195" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A195" s="24"/>
+    </row>
+    <row r="196" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A196" s="24"/>
+    </row>
+    <row r="197" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A197" s="24"/>
+    </row>
+    <row r="198" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A198" s="24"/>
+    </row>
+    <row r="199" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A199" s="24"/>
+    </row>
+    <row r="200" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A200" s="24"/>
+    </row>
+    <row r="201" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A201" s="24"/>
+    </row>
+    <row r="202" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A202" s="24"/>
+    </row>
+    <row r="203" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A203" s="24"/>
+    </row>
+    <row r="204" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A204" s="24"/>
+    </row>
+    <row r="205" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A205" s="24"/>
+    </row>
+    <row r="206" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A206" s="24"/>
+    </row>
+    <row r="207" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A207" s="24"/>
+    </row>
+    <row r="208" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A208" s="24"/>
+    </row>
+    <row r="209" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A209" s="24"/>
+    </row>
+    <row r="210" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A210" s="24"/>
+    </row>
+    <row r="211" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A211" s="24"/>
+    </row>
+    <row r="212" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A212" s="24"/>
+    </row>
+    <row r="213" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A213" s="24"/>
+    </row>
+    <row r="214" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A214" s="24"/>
+    </row>
+    <row r="215" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A215" s="24"/>
+    </row>
+    <row r="216" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A216" s="24"/>
+    </row>
+    <row r="217" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A217" s="24"/>
+    </row>
+    <row r="218" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A218" s="24"/>
+    </row>
+    <row r="219" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A219" s="24"/>
+    </row>
+    <row r="220" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A220" s="24"/>
+    </row>
+    <row r="221" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A221" s="24"/>
+    </row>
+    <row r="222" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A222" s="24"/>
+    </row>
+    <row r="223" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A223" s="24"/>
+    </row>
+    <row r="224" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A224" s="24"/>
+    </row>
+    <row r="225" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A225" s="24"/>
+    </row>
+    <row r="226" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A226" s="24"/>
+    </row>
+    <row r="227" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A227" s="24"/>
+    </row>
+    <row r="228" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A228" s="24"/>
+    </row>
+    <row r="229" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A229" s="24"/>
+    </row>
+    <row r="230" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A230" s="24"/>
+    </row>
+    <row r="231" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A231" s="24"/>
+    </row>
+    <row r="232" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A232" s="24"/>
+    </row>
+    <row r="233" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A233" s="24"/>
+    </row>
+    <row r="234" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A234" s="24"/>
+    </row>
+    <row r="235" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A235" s="24"/>
+    </row>
+    <row r="236" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A236" s="24"/>
+    </row>
+    <row r="237" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A237" s="24"/>
+    </row>
+    <row r="238" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A238" s="24"/>
+    </row>
+    <row r="239" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A239" s="24"/>
+    </row>
+    <row r="240" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A240" s="24"/>
+    </row>
+    <row r="241" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A241" s="24"/>
+    </row>
+    <row r="242" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A242" s="24"/>
+    </row>
+    <row r="243" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A243" s="24"/>
+    </row>
+    <row r="244" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A244" s="24"/>
+    </row>
+    <row r="245" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A245" s="24"/>
+    </row>
+    <row r="246" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A246" s="24"/>
+    </row>
+    <row r="247" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A247" s="24"/>
+    </row>
+    <row r="248" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A248" s="24"/>
+    </row>
+    <row r="249" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A249" s="24"/>
+    </row>
+    <row r="250" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A250" s="24"/>
+    </row>
+    <row r="251" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A251" s="24"/>
+    </row>
+    <row r="252" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A252" s="24"/>
+    </row>
+    <row r="253" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A253" s="24"/>
+    </row>
+    <row r="254" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A254" s="24"/>
+    </row>
+    <row r="255" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A255" s="24"/>
+    </row>
+    <row r="256" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A256" s="24"/>
+    </row>
+    <row r="257" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A257" s="24"/>
+    </row>
+    <row r="258" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A258" s="24"/>
+    </row>
+    <row r="259" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A259" s="24"/>
+    </row>
+    <row r="260" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A260" s="24"/>
+    </row>
+    <row r="261" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A261" s="24"/>
+    </row>
+    <row r="262" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A262" s="24"/>
+    </row>
+    <row r="263" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A263" s="24"/>
+    </row>
+    <row r="264" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A264" s="24"/>
+    </row>
+    <row r="265" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A265" s="24"/>
+    </row>
+    <row r="266" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A266" s="24"/>
+    </row>
+    <row r="267" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A267" s="24"/>
+    </row>
+    <row r="268" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A268" s="24"/>
+    </row>
+    <row r="269" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A269" s="24"/>
+    </row>
+    <row r="270" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A270" s="24"/>
+    </row>
+    <row r="271" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A271" s="24"/>
+    </row>
+    <row r="272" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A272" s="24"/>
+    </row>
+    <row r="273" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A273" s="24"/>
+    </row>
+    <row r="274" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A274" s="24"/>
+    </row>
+    <row r="275" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A275" s="24"/>
+    </row>
+    <row r="276" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A276" s="24"/>
+    </row>
+    <row r="277" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A277" s="24"/>
+    </row>
+    <row r="278" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A278" s="24"/>
+    </row>
+    <row r="279" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A279" s="24"/>
+    </row>
+    <row r="280" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A280" s="24"/>
+    </row>
+    <row r="281" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A281" s="24"/>
+    </row>
+    <row r="282" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A282" s="24"/>
+    </row>
+    <row r="283" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A283" s="24"/>
+    </row>
+    <row r="284" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A284" s="24"/>
+    </row>
+    <row r="285" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A285" s="24"/>
+    </row>
+    <row r="286" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A286" s="24"/>
+    </row>
+    <row r="287" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A287" s="24"/>
+    </row>
+    <row r="288" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A288" s="24"/>
+    </row>
+    <row r="289" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A289" s="24"/>
+    </row>
+    <row r="290" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A290" s="24"/>
+    </row>
+    <row r="291" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A291" s="24"/>
+    </row>
+    <row r="292" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A292" s="24"/>
+    </row>
+    <row r="293" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A293" s="24"/>
+    </row>
+    <row r="294" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A294" s="24"/>
+    </row>
+    <row r="295" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A295" s="24"/>
+    </row>
+    <row r="296" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A296" s="24"/>
+    </row>
+    <row r="297" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A297" s="24"/>
+    </row>
+    <row r="298" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A298" s="24"/>
+    </row>
+    <row r="299" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A299" s="24"/>
+    </row>
+    <row r="300" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A300" s="24"/>
+    </row>
+    <row r="301" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A301" s="24"/>
+    </row>
+    <row r="302" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A302" s="24"/>
+    </row>
+    <row r="303" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A303" s="24"/>
+    </row>
+    <row r="304" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A304" s="24"/>
+    </row>
+    <row r="305" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A305" s="24"/>
+    </row>
+    <row r="306" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A306" s="24"/>
+    </row>
+    <row r="307" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A307" s="24"/>
+    </row>
+    <row r="308" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A308" s="24"/>
+    </row>
+    <row r="309" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A309" s="24"/>
+    </row>
+    <row r="310" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A310" s="24"/>
+    </row>
+    <row r="311" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A311" s="24"/>
+    </row>
+    <row r="312" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A312" s="24"/>
+    </row>
+    <row r="313" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A313" s="24"/>
+    </row>
+    <row r="314" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A314" s="24"/>
+    </row>
+    <row r="315" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A315" s="24"/>
+    </row>
+    <row r="316" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A316" s="24"/>
+    </row>
+    <row r="317" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A317" s="24"/>
+    </row>
+    <row r="318" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A318" s="24"/>
+    </row>
+    <row r="319" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A319" s="24"/>
+    </row>
+    <row r="320" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A320" s="24"/>
+    </row>
+    <row r="321" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A321" s="24"/>
+    </row>
+    <row r="322" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A322" s="24"/>
+    </row>
+    <row r="323" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A323" s="24"/>
+    </row>
+    <row r="324" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A324" s="24"/>
+    </row>
+    <row r="325" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A325" s="24"/>
+    </row>
+    <row r="326" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A326" s="24"/>
+    </row>
+    <row r="327" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A327" s="24"/>
+    </row>
+    <row r="328" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A328" s="24"/>
+    </row>
+    <row r="329" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A329" s="24"/>
+    </row>
+    <row r="330" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A330" s="24"/>
+    </row>
+    <row r="331" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A331" s="24"/>
+    </row>
+    <row r="332" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A332" s="24"/>
+    </row>
+    <row r="333" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A333" s="24"/>
+    </row>
+    <row r="334" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A334" s="24"/>
+    </row>
+    <row r="335" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A335" s="24"/>
+    </row>
+    <row r="336" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A336" s="24"/>
+    </row>
+    <row r="337" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A337" s="24"/>
+    </row>
+    <row r="338" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A338" s="24"/>
+    </row>
+    <row r="339" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A339" s="24"/>
+    </row>
+    <row r="340" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A340" s="24"/>
+    </row>
+    <row r="341" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A341" s="24"/>
+    </row>
+    <row r="342" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A342" s="24"/>
+    </row>
+    <row r="343" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A343" s="24"/>
+    </row>
+    <row r="344" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A344" s="24"/>
+    </row>
+    <row r="345" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A345" s="24"/>
+    </row>
+    <row r="346" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A346" s="24"/>
+    </row>
+    <row r="347" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A347" s="24"/>
+    </row>
+    <row r="348" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A348" s="24"/>
+    </row>
+    <row r="349" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A349" s="24"/>
+    </row>
+    <row r="350" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A350" s="24"/>
+    </row>
+    <row r="351" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A351" s="24"/>
+    </row>
+    <row r="352" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A352" s="24"/>
+    </row>
+    <row r="353" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A353" s="24"/>
+    </row>
+    <row r="354" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A354" s="24"/>
+    </row>
+    <row r="355" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A355" s="24"/>
+    </row>
+    <row r="356" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A356" s="24"/>
+    </row>
+    <row r="357" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A357" s="24"/>
+    </row>
+    <row r="358" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A358" s="24"/>
+    </row>
+    <row r="359" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A359" s="24"/>
+    </row>
+    <row r="360" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A360" s="24"/>
+    </row>
+    <row r="361" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A361" s="24"/>
+    </row>
+    <row r="362" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A362" s="24"/>
+    </row>
+    <row r="363" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A363" s="24"/>
+    </row>
+    <row r="364" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A364" s="24"/>
+    </row>
+    <row r="365" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A365" s="24"/>
+    </row>
+    <row r="366" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A366" s="24"/>
+    </row>
+    <row r="367" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A367" s="24"/>
+    </row>
+    <row r="368" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A368" s="24"/>
+    </row>
+    <row r="369" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A369" s="24"/>
+    </row>
+    <row r="370" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A370" s="24"/>
+    </row>
+    <row r="371" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A371" s="24"/>
+    </row>
+    <row r="372" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A372" s="24"/>
+    </row>
+    <row r="373" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A373" s="24"/>
+    </row>
+    <row r="374" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A374" s="24"/>
+    </row>
+    <row r="375" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A375" s="24"/>
+    </row>
+    <row r="376" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A376" s="24"/>
+    </row>
+    <row r="377" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A377" s="24"/>
+    </row>
+    <row r="378" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A378" s="24"/>
+    </row>
+    <row r="379" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A379" s="24"/>
+    </row>
+    <row r="380" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A380" s="24"/>
+    </row>
+    <row r="381" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A381" s="24"/>
+    </row>
+    <row r="382" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A382" s="24"/>
+    </row>
+    <row r="383" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A383" s="24"/>
+    </row>
+    <row r="384" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A384" s="24"/>
+    </row>
+    <row r="385" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A385" s="24"/>
+    </row>
+    <row r="386" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A386" s="24"/>
+    </row>
+    <row r="387" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A387" s="24"/>
+    </row>
+    <row r="388" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A388" s="24"/>
+    </row>
+    <row r="389" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A389" s="24"/>
+    </row>
+    <row r="390" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A390" s="24"/>
+    </row>
+    <row r="391" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A391" s="24"/>
+    </row>
+    <row r="392" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A392" s="24"/>
+    </row>
+    <row r="393" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A393" s="24"/>
+    </row>
+    <row r="394" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A394" s="24"/>
+    </row>
+    <row r="395" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A395" s="24"/>
+    </row>
+    <row r="396" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A396" s="24"/>
+    </row>
+    <row r="397" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A397" s="24"/>
+    </row>
+    <row r="398" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A398" s="24"/>
+    </row>
+    <row r="399" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A399" s="24"/>
+    </row>
+    <row r="400" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A400" s="24"/>
+    </row>
+    <row r="401" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A401" s="24"/>
+    </row>
+    <row r="402" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A402" s="24"/>
+    </row>
+    <row r="403" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A403" s="24"/>
+    </row>
+    <row r="404" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A404" s="24"/>
+    </row>
+    <row r="405" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A405" s="24"/>
+    </row>
+    <row r="406" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A406" s="24"/>
+    </row>
+    <row r="407" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A407" s="24"/>
+    </row>
+    <row r="408" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A408" s="24"/>
+    </row>
+    <row r="409" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A409" s="24"/>
+    </row>
+    <row r="410" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A410" s="24"/>
+    </row>
+    <row r="411" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A411" s="24"/>
+    </row>
+    <row r="412" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A412" s="24"/>
+    </row>
+    <row r="413" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A413" s="24"/>
+    </row>
+    <row r="414" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A414" s="24"/>
+    </row>
+    <row r="415" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A415" s="24"/>
+    </row>
+    <row r="416" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A416" s="24"/>
+    </row>
+    <row r="417" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A417" s="24"/>
+    </row>
+    <row r="418" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A418" s="24"/>
+    </row>
+    <row r="419" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A419" s="24"/>
+    </row>
+    <row r="420" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A420" s="24"/>
+    </row>
+    <row r="421" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A421" s="24"/>
+    </row>
+    <row r="422" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A422" s="24"/>
+    </row>
+    <row r="423" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A423" s="24"/>
+    </row>
+    <row r="424" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A424" s="24"/>
+    </row>
+    <row r="425" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A425" s="24"/>
+    </row>
+    <row r="426" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A426" s="24"/>
+    </row>
+    <row r="427" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A427" s="24"/>
+    </row>
+    <row r="428" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A428" s="24"/>
+    </row>
+    <row r="429" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A429" s="24"/>
+    </row>
+    <row r="430" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A430" s="24"/>
+    </row>
+    <row r="431" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A431" s="24"/>
+    </row>
+    <row r="432" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A432" s="24"/>
+    </row>
+    <row r="433" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A433" s="24"/>
+    </row>
+    <row r="434" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A434" s="24"/>
+    </row>
+    <row r="435" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A435" s="24"/>
+    </row>
+    <row r="436" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A436" s="24"/>
+    </row>
+    <row r="437" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A437" s="24"/>
+    </row>
+    <row r="438" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A438" s="24"/>
+    </row>
+    <row r="439" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A439" s="24"/>
+    </row>
+    <row r="440" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A440" s="24"/>
+    </row>
+    <row r="441" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A441" s="24"/>
+    </row>
+    <row r="442" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A442" s="24"/>
+    </row>
+    <row r="443" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A443" s="24"/>
+    </row>
+    <row r="444" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A444" s="24"/>
+    </row>
+    <row r="445" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A445" s="24"/>
+    </row>
+    <row r="446" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A446" s="24"/>
+    </row>
+    <row r="447" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A447" s="24"/>
+    </row>
+    <row r="448" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A448" s="24"/>
+    </row>
+    <row r="449" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A449" s="24"/>
+    </row>
+    <row r="450" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A450" s="24"/>
+    </row>
+    <row r="451" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A451" s="24"/>
+    </row>
+    <row r="452" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A452" s="24"/>
+    </row>
+    <row r="453" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A453" s="24"/>
+    </row>
+    <row r="454" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A454" s="24"/>
+    </row>
+    <row r="455" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A455" s="24"/>
+    </row>
+    <row r="456" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A456" s="24"/>
+    </row>
+    <row r="457" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A457" s="24"/>
+    </row>
+    <row r="458" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A458" s="24"/>
+    </row>
+    <row r="459" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A459" s="24"/>
+    </row>
+    <row r="460" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A460" s="24"/>
+    </row>
+    <row r="461" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A461" s="24"/>
+    </row>
+    <row r="462" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A462" s="24"/>
+    </row>
+    <row r="463" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A463" s="24"/>
+    </row>
+    <row r="464" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A464" s="24"/>
+    </row>
+    <row r="465" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A465" s="24"/>
+    </row>
+    <row r="466" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A466" s="24"/>
+    </row>
+    <row r="467" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A467" s="24"/>
+    </row>
+    <row r="468" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A468" s="24"/>
+    </row>
+    <row r="469" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A469" s="24"/>
+    </row>
+    <row r="470" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A470" s="24"/>
+    </row>
+    <row r="471" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A471" s="24"/>
+    </row>
+    <row r="472" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A472" s="24"/>
+    </row>
+    <row r="473" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A473" s="24"/>
+    </row>
+    <row r="474" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A474" s="24"/>
+    </row>
+    <row r="475" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A475" s="24"/>
+    </row>
+    <row r="476" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A476" s="24"/>
+    </row>
+    <row r="477" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A477" s="24"/>
+    </row>
+    <row r="478" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A478" s="24"/>
+    </row>
+    <row r="479" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A479" s="24"/>
+    </row>
+    <row r="480" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A480" s="24"/>
+    </row>
+    <row r="481" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A481" s="24"/>
+    </row>
+    <row r="482" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A482" s="24"/>
+    </row>
+    <row r="483" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A483" s="24"/>
+    </row>
+    <row r="484" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A484" s="24"/>
+    </row>
+    <row r="485" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A485" s="24"/>
+    </row>
+    <row r="486" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A486" s="24"/>
+    </row>
+    <row r="487" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A487" s="24"/>
+    </row>
+    <row r="488" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A488" s="24"/>
+    </row>
+    <row r="489" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A489" s="24"/>
+    </row>
+    <row r="490" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A490" s="24"/>
+    </row>
+    <row r="491" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A491" s="24"/>
+    </row>
+    <row r="492" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A492" s="24"/>
+    </row>
+    <row r="493" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A493" s="24"/>
+    </row>
+    <row r="494" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A494" s="24"/>
+    </row>
+    <row r="495" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A495" s="24"/>
+    </row>
+    <row r="496" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A496" s="24"/>
+    </row>
+    <row r="497" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A497" s="24"/>
+    </row>
+    <row r="498" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A498" s="24"/>
+    </row>
+    <row r="499" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A499" s="24"/>
+    </row>
+    <row r="500" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A500" s="24"/>
+    </row>
+    <row r="501" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A501" s="24"/>
+    </row>
+    <row r="502" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A502" s="24"/>
+    </row>
+    <row r="503" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A503" s="24"/>
+    </row>
+    <row r="504" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A504" s="24"/>
+    </row>
+    <row r="505" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A505" s="24"/>
+    </row>
+    <row r="506" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A506" s="24"/>
+    </row>
+    <row r="507" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A507" s="24"/>
+    </row>
+    <row r="508" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A508" s="24"/>
+    </row>
+    <row r="509" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A509" s="24"/>
+    </row>
+    <row r="510" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A510" s="24"/>
+    </row>
+    <row r="511" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A511" s="24"/>
+    </row>
+    <row r="512" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A512" s="24"/>
+    </row>
+    <row r="513" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A513" s="24"/>
+    </row>
+    <row r="514" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A514" s="24"/>
+    </row>
+    <row r="515" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A515" s="24"/>
+    </row>
+    <row r="516" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A516" s="24"/>
+    </row>
+    <row r="517" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A517" s="24"/>
+    </row>
+    <row r="518" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A518" s="24"/>
+    </row>
+    <row r="519" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A519" s="24"/>
+    </row>
+    <row r="520" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A520" s="24"/>
+    </row>
+    <row r="521" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A521" s="24"/>
+    </row>
+    <row r="522" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A522" s="24"/>
+    </row>
+    <row r="523" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A523" s="24"/>
+    </row>
+    <row r="524" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A524" s="24"/>
+    </row>
+    <row r="525" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A525" s="24"/>
+    </row>
+    <row r="526" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A526" s="24"/>
+    </row>
+    <row r="527" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A527" s="24"/>
+    </row>
+    <row r="528" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A528" s="24"/>
+    </row>
+    <row r="529" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A529" s="24"/>
+    </row>
+    <row r="530" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A530" s="24"/>
+    </row>
+    <row r="531" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A531" s="24"/>
+    </row>
+    <row r="532" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A532" s="24"/>
+    </row>
+    <row r="533" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A533" s="24"/>
+    </row>
+    <row r="534" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A534" s="24"/>
+    </row>
+    <row r="535" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A535" s="24"/>
+    </row>
+    <row r="536" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A536" s="24"/>
+    </row>
+    <row r="537" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A537" s="24"/>
+    </row>
+    <row r="538" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A538" s="24"/>
+    </row>
+    <row r="539" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A539" s="24"/>
+    </row>
+    <row r="540" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A540" s="24"/>
+    </row>
+    <row r="541" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A541" s="24"/>
+    </row>
+    <row r="542" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A542" s="24"/>
+    </row>
+    <row r="543" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A543" s="24"/>
+    </row>
+    <row r="544" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A544" s="24"/>
+    </row>
+    <row r="545" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A545" s="24"/>
+    </row>
+    <row r="546" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A546" s="24"/>
+    </row>
+    <row r="547" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A547" s="24"/>
+    </row>
+    <row r="548" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A548" s="24"/>
+    </row>
+    <row r="549" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A549" s="24"/>
+    </row>
+    <row r="550" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A550" s="24"/>
+    </row>
+    <row r="551" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A551" s="24"/>
+    </row>
+    <row r="552" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A552" s="24"/>
+    </row>
+    <row r="553" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A553" s="24"/>
+    </row>
+    <row r="554" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A554" s="24"/>
+    </row>
+    <row r="555" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A555" s="24"/>
+    </row>
+    <row r="556" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A556" s="24"/>
+    </row>
+    <row r="557" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A557" s="24"/>
+    </row>
+    <row r="558" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A558" s="24"/>
+    </row>
+    <row r="559" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A559" s="24"/>
+    </row>
+    <row r="560" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A560" s="24"/>
+    </row>
+    <row r="561" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A561" s="24"/>
+    </row>
+    <row r="562" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A562" s="24"/>
+    </row>
+    <row r="563" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A563" s="24"/>
+    </row>
+    <row r="564" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A564" s="24"/>
+    </row>
+    <row r="565" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A565" s="24"/>
+    </row>
+    <row r="566" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A566" s="24"/>
+    </row>
+    <row r="567" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A567" s="24"/>
+    </row>
+    <row r="568" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A568" s="24"/>
+    </row>
+    <row r="569" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A569" s="24"/>
+    </row>
+    <row r="570" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A570" s="24"/>
+    </row>
+    <row r="571" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A571" s="24"/>
+    </row>
+    <row r="572" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A572" s="24"/>
+    </row>
+    <row r="573" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A573" s="24"/>
+    </row>
+    <row r="574" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A574" s="24"/>
+    </row>
+    <row r="575" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A575" s="24"/>
+    </row>
+    <row r="576" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A576" s="24"/>
+    </row>
+    <row r="577" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A577" s="24"/>
+    </row>
+    <row r="578" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A578" s="24"/>
+    </row>
+    <row r="579" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A579" s="24"/>
+    </row>
+    <row r="580" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A580" s="24"/>
+    </row>
+    <row r="581" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A581" s="24"/>
+    </row>
+    <row r="582" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A582" s="24"/>
+    </row>
+    <row r="583" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A583" s="24"/>
+    </row>
+    <row r="584" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A584" s="24"/>
+    </row>
+    <row r="585" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A585" s="24"/>
+    </row>
+    <row r="586" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A586" s="24"/>
+    </row>
+    <row r="587" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A587" s="24"/>
+    </row>
+    <row r="588" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A588" s="24"/>
+    </row>
+    <row r="589" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A589" s="24"/>
+    </row>
+    <row r="590" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A590" s="24"/>
+    </row>
+    <row r="591" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A591" s="24"/>
+    </row>
+    <row r="592" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A592" s="24"/>
+    </row>
+    <row r="593" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A593" s="24"/>
+    </row>
+    <row r="594" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A594" s="24"/>
+    </row>
+    <row r="595" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A595" s="24"/>
+    </row>
+    <row r="596" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A596" s="24"/>
+    </row>
+    <row r="597" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A597" s="24"/>
+    </row>
+    <row r="598" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A598" s="24"/>
+    </row>
+    <row r="599" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A599" s="24"/>
+    </row>
+    <row r="600" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A600" s="24"/>
+    </row>
+    <row r="601" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A601" s="24"/>
+    </row>
+    <row r="602" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A602" s="24"/>
+    </row>
+    <row r="603" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A603" s="24"/>
+    </row>
+    <row r="604" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A604" s="24"/>
+    </row>
+    <row r="605" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A605" s="24"/>
+    </row>
+    <row r="606" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A606" s="24"/>
+    </row>
+    <row r="607" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A607" s="24"/>
+    </row>
+    <row r="608" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A608" s="24"/>
+    </row>
+    <row r="609" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A609" s="24"/>
+    </row>
+    <row r="610" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A610" s="24"/>
+    </row>
+    <row r="611" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A611" s="24"/>
+    </row>
+    <row r="612" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A612" s="24"/>
+    </row>
+    <row r="613" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A613" s="24"/>
+    </row>
+    <row r="614" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A614" s="24"/>
+    </row>
+    <row r="615" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A615" s="24"/>
+    </row>
+    <row r="616" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A616" s="24"/>
+    </row>
+    <row r="617" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A617" s="24"/>
+    </row>
+    <row r="618" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A618" s="24"/>
+    </row>
+    <row r="619" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A619" s="24"/>
+    </row>
+    <row r="620" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A620" s="24"/>
+    </row>
+    <row r="621" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A621" s="24"/>
+    </row>
+    <row r="622" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A622" s="24"/>
+    </row>
+    <row r="623" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A623" s="24"/>
+    </row>
+    <row r="624" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A624" s="24"/>
+    </row>
+    <row r="625" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A625" s="24"/>
+    </row>
+    <row r="626" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A626" s="24"/>
+    </row>
+    <row r="627" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A627" s="24"/>
+    </row>
+    <row r="628" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A628" s="24"/>
+    </row>
+    <row r="629" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A629" s="24"/>
+    </row>
+    <row r="630" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A630" s="24"/>
+    </row>
+    <row r="631" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A631" s="24"/>
+    </row>
+    <row r="632" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A632" s="24"/>
+    </row>
+    <row r="633" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A633" s="24"/>
+    </row>
+    <row r="634" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A634" s="24"/>
+    </row>
+    <row r="635" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A635" s="24"/>
+    </row>
+    <row r="636" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A636" s="24"/>
+    </row>
+    <row r="637" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A637" s="24"/>
+    </row>
+    <row r="638" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A638" s="24"/>
+    </row>
+    <row r="639" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A639" s="24"/>
+    </row>
+    <row r="640" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A640" s="24"/>
+    </row>
+    <row r="641" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A641" s="24"/>
+    </row>
+    <row r="642" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A642" s="24"/>
+    </row>
+    <row r="643" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A643" s="24"/>
+    </row>
+    <row r="644" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A644" s="24"/>
+    </row>
+    <row r="645" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A645" s="24"/>
+    </row>
+    <row r="646" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A646" s="24"/>
+    </row>
+    <row r="647" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A647" s="24"/>
+    </row>
+    <row r="648" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A648" s="24"/>
+    </row>
+    <row r="649" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A649" s="24"/>
+    </row>
+    <row r="650" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A650" s="24"/>
+    </row>
+    <row r="651" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A651" s="24"/>
+    </row>
+    <row r="652" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A652" s="24"/>
+    </row>
+    <row r="653" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A653" s="24"/>
+    </row>
+    <row r="654" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A654" s="24"/>
+    </row>
+    <row r="655" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A655" s="24"/>
+    </row>
+    <row r="656" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A656" s="24"/>
+    </row>
+    <row r="657" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A657" s="24"/>
+    </row>
+    <row r="658" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A658" s="24"/>
+    </row>
+    <row r="659" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A659" s="24"/>
+    </row>
+    <row r="660" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A660" s="24"/>
+    </row>
+    <row r="661" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A661" s="24"/>
+    </row>
+    <row r="662" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A662" s="24"/>
+    </row>
+    <row r="663" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A663" s="24"/>
+    </row>
+    <row r="664" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A664" s="24"/>
+    </row>
+    <row r="665" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A665" s="24"/>
+    </row>
+    <row r="666" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A666" s="24"/>
+    </row>
+    <row r="667" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A667" s="24"/>
+    </row>
+    <row r="668" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A668" s="24"/>
+    </row>
+    <row r="669" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A669" s="24"/>
+    </row>
+    <row r="670" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A670" s="24"/>
+    </row>
+    <row r="671" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A671" s="24"/>
+    </row>
+    <row r="672" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A672" s="24"/>
+    </row>
+    <row r="673" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A673" s="24"/>
+    </row>
+    <row r="674" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A674" s="24"/>
+    </row>
+    <row r="675" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A675" s="24"/>
+    </row>
+    <row r="676" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A676" s="24"/>
+    </row>
+    <row r="677" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A677" s="24"/>
+    </row>
+    <row r="678" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A678" s="24"/>
+    </row>
+    <row r="679" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A679" s="24"/>
+    </row>
+    <row r="680" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A680" s="24"/>
+    </row>
+    <row r="681" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A681" s="24"/>
+    </row>
+    <row r="682" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A682" s="24"/>
+    </row>
+    <row r="683" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A683" s="24"/>
+    </row>
+    <row r="684" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A684" s="24"/>
+    </row>
+    <row r="685" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A685" s="25"/>
+    </row>
+    <row r="686" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A686" s="25"/>
+    </row>
+    <row r="687" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A687" s="25"/>
+    </row>
+    <row r="688" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A688" s="25"/>
+    </row>
+    <row r="689" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A689" s="25"/>
+    </row>
+    <row r="690" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A690" s="25"/>
+    </row>
+    <row r="691" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A691" s="25"/>
+    </row>
+    <row r="692" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A692" s="25"/>
+    </row>
+    <row r="693" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A693" s="25"/>
+    </row>
+    <row r="694" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A694" s="25"/>
+    </row>
+    <row r="695" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A695" s="25"/>
+    </row>
+    <row r="696" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A696" s="25"/>
+    </row>
+    <row r="697" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A697" s="25"/>
+    </row>
+    <row r="698" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A698" s="25"/>
+    </row>
+    <row r="699" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A699" s="25"/>
+    </row>
+    <row r="700" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A700" s="25"/>
+    </row>
+    <row r="701" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A701" s="25"/>
+    </row>
+    <row r="702" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A702" s="25"/>
+    </row>
+    <row r="703" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A703" s="25"/>
+    </row>
+    <row r="704" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A704" s="25"/>
+    </row>
+    <row r="705" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A705" s="25"/>
+    </row>
+    <row r="706" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A706" s="25"/>
+    </row>
+    <row r="707" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A707" s="25"/>
+    </row>
+    <row r="708" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A708" s="25"/>
+    </row>
+    <row r="709" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A709" s="25"/>
+    </row>
+    <row r="710" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A710" s="25"/>
+    </row>
+    <row r="711" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A711" s="25"/>
+    </row>
+    <row r="712" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A712" s="25"/>
+    </row>
+    <row r="713" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A713" s="25"/>
+    </row>
+    <row r="714" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A714" s="25"/>
+    </row>
+    <row r="715" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A715" s="25"/>
+    </row>
+    <row r="716" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A716" s="25"/>
+    </row>
+    <row r="717" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A717" s="25"/>
+    </row>
+    <row r="718" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A718" s="25"/>
+    </row>
+    <row r="719" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A719" s="25"/>
+    </row>
+    <row r="720" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A720" s="25"/>
+    </row>
+    <row r="721" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A721" s="25"/>
+    </row>
+    <row r="722" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A722" s="25"/>
+    </row>
+    <row r="723" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A723" s="25"/>
+    </row>
+    <row r="724" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A724" s="25"/>
+    </row>
+    <row r="725" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A725" s="25"/>
+    </row>
+    <row r="726" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A726" s="25"/>
+    </row>
+    <row r="727" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A727" s="25"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Atualização dos dados de produção
</commit_message>
<xml_diff>
--- a/DadosProducao.xlsx
+++ b/DadosProducao.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\AcompanhamentoProducao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D347B0F8-E786-4F3C-9C1F-6E46E18E9168}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B1FAB18-44D2-4ADA-B1F9-7FFBBB5AEF72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{3AA6C56D-DA97-499B-A05C-D9170B04DAB1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{3AA6C56D-DA97-499B-A05C-D9170B04DAB1}"/>
   </bookViews>
   <sheets>
     <sheet name="DadosBrutos" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1361,86 +1361,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="11">
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <gradientFill degree="90">
-          <stop position="0">
-            <color rgb="FFFF33CC"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FF8F098C"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-      <fill>
-        <gradientFill degree="90">
-          <stop position="0">
-            <color rgb="FF35DFCF"/>
-          </stop>
-          <stop position="1">
-            <color rgb="FF92D050"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF32FC00"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF00B0F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFC000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="5">
     <dxf>
       <font>
         <b/>
@@ -1526,10 +1447,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -35046,19 +34963,19 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A1">
-    <cfRule type="duplicateValues" dxfId="10" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F1">
-    <cfRule type="containsText" dxfId="9" priority="3" operator="containsText" text="MATERIAL FALTANDO">
+    <cfRule type="containsText" dxfId="3" priority="3" operator="containsText" text="MATERIAL FALTANDO">
       <formula>NOT(ISERROR(SEARCH("MATERIAL FALTANDO",F1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="8" priority="5" operator="containsText" text="FATURADO">
+    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="FATURADO">
       <formula>NOT(ISERROR(SEARCH("FATURADO",F1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="7" priority="6" operator="containsText" text="CONFERIDO">
+    <cfRule type="containsText" dxfId="1" priority="6" operator="containsText" text="CONFERIDO">
       <formula>NOT(ISERROR(SEARCH("CONFERIDO",F1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="SEPARANDO">
+    <cfRule type="containsText" dxfId="0" priority="7" operator="containsText" text="SEPARANDO">
       <formula>NOT(ISERROR(SEARCH("SEPARANDO",F1)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -35077,7 +34994,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="str" cm="1">
-        <f t="array" ref="A1:A19">_xlfn.UNIQUE(DadosBrutos!C1:C1159)</f>
+        <f t="array" ref="A1:A20">_xlfn.UNIQUE(DadosBrutos!C1:C1273)</f>
         <v>DATA</v>
       </c>
       <c r="B1" s="19" t="s">
@@ -35247,7 +35164,13 @@
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="20"/>
+      <c r="A20" s="20">
+        <v>46322</v>
+      </c>
+      <c r="B20" s="18">
+        <f>COUNTIF(DadosBrutos!C:C, A20)</f>
+        <v>27</v>
+      </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="20"/>
@@ -37388,7 +37311,7 @@
   <sheetData>
     <row r="1" spans="1:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="str" cm="1">
-        <f t="array" ref="A1:A19">_xlfn.UNIQUE(DadosBrutos!C1:C1159)</f>
+        <f t="array" ref="A1:A20">_xlfn.UNIQUE(DadosBrutos!C1:C1273)</f>
         <v>DATA</v>
       </c>
       <c r="B1" s="19" t="s">
@@ -37633,7 +37556,17 @@
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="20"/>
+      <c r="A20" s="20">
+        <v>46322</v>
+      </c>
+      <c r="B20">
+        <f>COUNTIFS(DadosBrutos!C:C, A20, DadosBrutos!G:G, "SAUDAVEL")</f>
+        <v>0</v>
+      </c>
+      <c r="C20">
+        <f>COUNTIFS(DadosBrutos!C:C, A20, DadosBrutos!G:G, "BACKLOG")</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="20"/>

</xml_diff>